<commit_message>
ORFS: 29 more Brennan STEPs filed; loose parts at every size (FS0306 / FS0318 / FS0319 / FS0319C)
- 09_STEP_FILES: per-size nut / sleeve STEPs, FS6500-04 ... -20, FS2403-24-24, FS6400-32-32-O,
  FS2501-08-08-FG, FS6565-08-08 (sha256 in tools/_out/orfs_steps2_20261020)
- staging gen_straight2: per-size countersink / nut / sleeve measurements, the coned-collar
  sleeve (-12 / -16 / -20) as master FS0319C; Brennan's smaller -10 / -24 nut thread bores
  noted in the rows' COMMENT (model keeps the basic minor)
- 22 loose configurations: static checks clean, OCP closed loop 427 checks 0 off,
  regression 99 / 99 identical

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QQuceHR8ZUuy6411Z8yX1P
</commit_message>
<xml_diff>
--- a/tools/_out/orfs_gen_20261020/out/DesignTable_FS0306_SW2.xlsx
+++ b/tools/_out/orfs_gen_20261020/out/DesignTable_FS0306_SW2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -621,7 +621,7 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Air-Way FF306 (s3, double-pass 2026-10-15, parts.air-way.com/api/series/3, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p20 FS0306-08 (ORFS-p020-t01) | MODEL: face-seal bulkhead locknut (Brennan FS0306-08): hex S4 / thickness h2 = Air-Way; thread = the face-seal thread of the dash through, minor = ASME B1.1 basic minor; 45deg countersink on both faces from the minor to r 0.4095 measured on the -08 pilot (other sizes need their own STEP); hex end chamfers (75deg) NOT modelled; single manufacturer</t>
+          <t>Air-Way FF306 (s3, double-pass 2026-10-15, parts.air-way.com/api/series/3, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p20 FS0306-08 (ORFS-p020-t01) | MODEL: face-seal bulkhead locknut (Brennan FS0306-08): hex S4 / thickness h2 = the row; thread = the face-seal thread of the dash through, minor = ASME B1.1 basic minor; 45deg countersink on both faces from the minor to r 0.4095 measured on BRENNAN_FS0306-08 (tools/_out/orfs_steps2_20261020/loose_survey.txt (-08: tools/_out/orfs_wp2_20261020/end_lib_08.json)); hex end chamfers (75deg) NOT modelled; single manufacturer</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -632,6 +632,685 @@
       <c r="Y2" t="inlineStr">
         <is>
           <t>FS0306-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FS0306-04</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.46881</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.25118</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.2805</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.2805</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.25118</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.50236</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.05556</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.25118</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.28125</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.50236</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>FS0306-04</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>ORFS Bulkhead Locknut, 9/16-18 UN-2B, thread through, 45 deg countersink both faces</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>FS0306</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>9/16-18 UN (45deg countersink)</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>9/16-18 UN-2B (face-seal locknut thread, through)</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row (FF306 has no row of this size) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): H2@DRIVE: Brennan ORFS catalog p20 table ORFS-p020-t01 "FS0306 BULKHEAD LOCK NUT" row FS0306-04 col "TT WIDTH" = "0.270" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 196.9, page verified True) [Brennan = yes 2026-10-18] - nut thickness; mapping: same-table check: 6/6 rows with an Air-Way value agree to rounding; S4HEX@HEX: Brennan ORFS catalog p20 table ORFS-p020-t01 "FS0306 BULKHEAD LOCK NUT" row FS0306-04 col "B HEX" = "0.812" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 196.9, page verified True) [Brennan = yes 2026-10-18] - nut hex; mapping: same-table check: 6/6 rows with an Air-Way value agree to rounding; THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -04 = 0.5625 (PLAN.md s2 FS_THR / the -04 thread of every staged ORFS row); = Brennan "A THREAD" "9/16-18" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p20 table ORFS-p020-t01 "FS0306 BULKHEAD LOCK NUT" row FS0306-04 col "A THREAD" "9/16-18" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p20 table ORFS-p020-t01 "FS0306 BULKHEAD LOCK NUT" row FS0306-04 col "TUBE O.D." "1/4" in the table's format | MODEL: face-seal bulkhead locknut (Brennan FS0306-04): hex S4 / thickness h2 = the row; thread = the face-seal thread of the dash through, minor = ASME B1.1 basic minor; 45deg countersink on both faces from the minor to r 0.2805 measured on BRENNAN_FS0306-04 (tools/_out/orfs_steps2_20261020/loose_survey.txt (-08: tools/_out/orfs_wp2_20261020/end_lib_08.json)); hex end chamfers (75deg) NOT modelled; single manufacturer</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>no Air-Way FF306 row of this size (Brennan prints it: Brennan-only stays MISSING) | OMi parts file row 5215 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p20 FS0306-04 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>FS0306-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FS0306-06</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.57735</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.30992</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.3465</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.3465</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.30992</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.6198399999999999</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.30992</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.34375</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.6198399999999999</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>FS0306-06</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>ORFS Bulkhead Locknut, 11/16-16 UN-2B, thread through, 45 deg countersink both faces</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>FS0306</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>11/16-16 UN (45deg countersink)</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>11/16-16 UN-2B (face-seal locknut thread, through)</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 (s3, double-pass 2026-10-15, parts.air-way.com/api/series/3, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p20 FS0306-06 (ORFS-p020-t01) | MODEL: face-seal bulkhead locknut (Brennan FS0306-06): hex S4 / thickness h2 = the row; thread = the face-seal thread of the dash through, minor = ASME B1.1 basic minor; 45deg countersink on both faces from the minor to r 0.3465 measured on BRENNAN_FS0306-06 (tools/_out/orfs_steps2_20261020/loose_survey.txt (-08: tools/_out/orfs_wp2_20261020/end_lib_08.json)); hex end chamfers (75deg) NOT modelled; single manufacturer</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 = Brennan p20 on nut width, hex (rounding-only differences count as equal) | OMi parts file row 5216 (no dimensions) | DataStatus VERIFIED -&gt; ASSUMED: the face-seal end shapes are measured on Brennan STEPs only (Air-Way 3D models not yet measured)</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>FS0306-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FS0306-10</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.7563299999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.46134</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.46134</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.9226799999999999</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.07142999999999999</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.46134</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.9226799999999999</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>FS0306-10</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>ORFS Bulkhead Locknut, 1-14 UN-2B, thread through, 45 deg countersink both faces</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>FS0306</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>1-14 UN (45deg countersink)</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>1-14 UN-2B (face-seal locknut thread, through)</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 (s3, double-pass 2026-10-15, parts.air-way.com/api/series/3, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p20 FS0306-10 (ORFS-p020-t01) | MODEL: face-seal bulkhead locknut (Brennan FS0306-10): hex S4 / thickness h2 = the row; thread = the face-seal thread of the dash through, minor = ASME B1.1 basic minor; 45deg countersink on both faces from the minor to r 0.502 measured on BRENNAN_FS0306-10 (tools/_out/orfs_steps2_20261020/loose_survey.txt (-08: tools/_out/orfs_wp2_20261020/end_lib_08.json)); hex end chamfers (75deg) NOT modelled; single manufacturer</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 = Brennan p20 on nut width, hex (rounding-only differences count as equal) | OMi parts file row 5218 (no dimensions) | BRENNAN DIFFERS: BRENNAN_FS0306-10 has its thread bore at dia 0.8920; the model uses the ASME B1.1 basic minor 0.9227 of 1-14 (the thread of the row) - tell the user; DataStatus VERIFIED -&gt; ASSUMED: the face-seal end shapes are measured on Brennan STEPs only (Air-Way 3D models not yet measured)</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>FS0306-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FS0306-12</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.86603</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.54864</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.5965</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.5965</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.54864</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1.09728</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.54864</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.59375</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1.09728</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>FS0306-12</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>ORFS Bulkhead Locknut, 1 3/16-12 UN-2B, thread through, 45 deg countersink both faces</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>FS0306</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>1 3/16-12 UN (45deg countersink)</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>1 3/16-12 UN-2B (face-seal locknut thread, through)</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>[BRENNAN-ONLY 2026-10-18] no Air-Way row (FF306 has no row of this size) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): H2@DRIVE: Brennan ORFS catalog p20 table ORFS-p020-t01 "FS0306 BULKHEAD LOCK NUT" row FS0306-12 col "TT WIDTH" = "0.410" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 237.2, page verified True) [Brennan = yes 2026-10-18] - nut thickness; mapping: same-table check: 6/6 rows with an Air-Way value agree to rounding; S4HEX@HEX: Brennan ORFS catalog p20 table ORFS-p020-t01 "FS0306 BULKHEAD LOCK NUT" row FS0306-12 col "B HEX" = "1.500" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 237.2, page verified True) [Brennan = yes 2026-10-18] - nut hex; mapping: same-table check: 6/6 rows with an Air-Way value agree to rounding; THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -12 = 1.1875 (PLAN.md s2 FS_THR / the -12 thread of every staged ORFS row); = Brennan "A THREAD" "1-3/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p20 table ORFS-p020-t01 "FS0306 BULKHEAD LOCK NUT" row FS0306-12 col "A THREAD" "1-3/16-12" in the table's format; $PRP@TubeOD: Brennan ORFS catalog p20 table ORFS-p020-t01 "FS0306 BULKHEAD LOCK NUT" row FS0306-12 col "TUBE O.D." "3/4" in the table's format | MODEL: face-seal bulkhead locknut (Brennan FS0306-12): hex S4 / thickness h2 = the row; thread = the face-seal thread of the dash through, minor = ASME B1.1 basic minor; 45deg countersink on both faces from the minor to r 0.5965 measured on BRENNAN_FS0306-12 (tools/_out/orfs_steps2_20261020/loose_survey.txt (-08: tools/_out/orfs_wp2_20261020/end_lib_08.json)); hex end chamfers (75deg) NOT modelled; single manufacturer</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>no Air-Way FF306 row of this size (Brennan prints it: Brennan-only stays MISSING) | OMi parts file row 5219 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p20 FS0306-12 ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>FS0306-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FS0306-16</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.01036</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.67364</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.7205</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.7205</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.67364</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1.34728</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.67364</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.71875</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1.34728</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>FS0306-16</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>ORFS Bulkhead Locknut, 1 7/16-12 UN-2B, thread through, 45 deg countersink both faces</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>FS0306</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>1 7/16-12 UN (45deg countersink)</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>1 7/16-12 UN-2B (face-seal locknut thread, through)</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 (s3, double-pass 2026-10-15, parts.air-way.com/api/series/3, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p20 FS0306-16 (ORFS-p020-t01) | MODEL: face-seal bulkhead locknut (Brennan FS0306-16): hex S4 / thickness h2 = the row; thread = the face-seal thread of the dash through, minor = ASME B1.1 basic minor; 45deg countersink on both faces from the minor to r 0.7205 measured on BRENNAN_FS0306-16 (tools/_out/orfs_steps2_20261020/loose_survey.txt (-08: tools/_out/orfs_wp2_20261020/end_lib_08.json)); hex end chamfers (75deg) NOT modelled; single manufacturer</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 = Brennan p20 on nut width, hex (rounding-only differences count as equal) | OMi parts file row 5220 (no dimensions) | DataStatus VERIFIED -&gt; ASSUMED: the face-seal end shapes are measured on Brennan STEPs only (Air-Way 3D models not yet measured)</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>FS0306-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FS0306-20</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.1547</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.79864</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.8465</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.8465</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.79864</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.59728</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.79864</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.84375</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1.59728</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>FS0306-20</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>ORFS Bulkhead Locknut, 1 11/16-12 UN-2B, thread through, 45 deg countersink both faces</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>FS0306</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>1 11/16-12 UN (45deg countersink)</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>1 11/16-12 UN-2B (face-seal locknut thread, through)</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 (s3, double-pass 2026-10-15, parts.air-way.com/api/series/3, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p20 FS0306-20 (ORFS-p020-t01) | MODEL: face-seal bulkhead locknut (Brennan FS0306-20): hex S4 / thickness h2 = the row; thread = the face-seal thread of the dash through, minor = ASME B1.1 basic minor; 45deg countersink on both faces from the minor to r 0.8465 measured on BRENNAN_FS0306-20 (tools/_out/orfs_steps2_20261020/loose_survey.txt (-08: tools/_out/orfs_wp2_20261020/end_lib_08.json)); hex end chamfers (75deg) NOT modelled; single manufacturer</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 = Brennan p20 on nut width, hex (rounding-only differences count as equal) | OMi parts file row 5221 (no dimensions) | DataStatus VERIFIED -&gt; ASSUMED: the face-seal end shapes are measured on Brennan STEPs only (Air-Way 3D models not yet measured)</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>FS0306-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FS0306-24</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.37409</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.95489</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.002</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.002</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.95489</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.90978</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.08333</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.95489</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1.90978</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>FS0306-24</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>ORFS Bulkhead Locknut, 2-12 UN-2B, thread through, 45 deg countersink both faces</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>FS0306</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>2-12 UN (45deg countersink)</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>2-12 UN-2B (face-seal locknut thread, through)</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 (s3, double-pass 2026-10-15, parts.air-way.com/api/series/3, two fetches identical) [user 2026-10-15: "use airway dimensions, check brennan too"]; checked against the Brennan ORFS catalog p20 FS0306-24 (ORFS-p020-t01) | MODEL: face-seal bulkhead locknut (Brennan FS0306-24): hex S4 / thickness h2 = the row; thread = the face-seal thread of the dash through, minor = ASME B1.1 basic minor; 45deg countersink on both faces from the minor to r 1.002 measured on BRENNAN_FS0306-24 (tools/_out/orfs_steps2_20261020/loose_survey.txt (-08: tools/_out/orfs_wp2_20261020/end_lib_08.json)); hex end chamfers (75deg) NOT modelled; single manufacturer</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Air-Way FF306 = Brennan p20 on nut width, hex (rounding-only differences count as equal) | OMi parts file row 5222 (no dimensions) | BRENNAN DIFFERS: BRENNAN_FS0306-24 has its thread bore at dia 1.8170; the model uses the ASME B1.1 basic minor 1.9098 of 2-12 (the thread of the row) - tell the user; DataStatus VERIFIED -&gt; ASSUMED: the face-seal end shapes are measured on Brennan STEPs only (Air-Way 3D models not yet measured)</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>FS0306-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PC: ORFS staging regenerated locally 2026-10-20
</commit_message>
<xml_diff>
--- a/tools/_out/orfs_gen_20261020/out/DesignTable_FS0306_SW2.xlsx
+++ b/tools/_out/orfs_gen_20261020/out/DesignTable_FS0306_SW2.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>